<commit_message>
feat: complete take-home test with clean output, multi-email, and robust matching
</commit_message>
<xml_diff>
--- a/output/Working_Paper_Result.xlsx
+++ b/output/Working_Paper_Result.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Working_Paper_Result" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Working_Paper_Result" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -87,17 +87,17 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="002D3748"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001A365D"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="002D3748"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -126,6 +126,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="002B6CB0"/>
         <bgColor rgb="002B6CB0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF2F7"/>
+        <bgColor rgb="00EDF2F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -421,7 +427,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -537,8 +543,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -814,18 +825,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" style="31" min="1" max="1"/>
-    <col width="25" customWidth="1" style="31" min="2" max="2"/>
-    <col width="15" customWidth="1" style="31" min="3" max="3"/>
-    <col width="20" customWidth="1" style="31" min="4" max="4"/>
-    <col width="20" customWidth="1" style="31" min="5" max="5"/>
-    <col width="22" customWidth="1" style="31" min="6" max="6"/>
-    <col width="22" customWidth="1" style="31" min="7" max="7"/>
-    <col width="15" customWidth="1" style="31" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="31">
       <c r="A1" s="49" t="inlineStr">
@@ -954,311 +955,293 @@
     <row r="13">
       <c r="B13" s="54" t="inlineStr">
         <is>
-          <t>EXECUTIVE SUMMARY (AI GENERATED)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
+          <t>EXECUTIVE SUMMARY (LAPORAN REKONSILIASI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="31">
       <c r="B15" s="57" t="inlineStr">
         <is>
-          <t>Tentu, berikut adalah Executive Summary profesional dan ringkas mengenai hasil rekonsiliasi Advance Settlement periode April 2026 untuk Direksi PT. Setiawan Dwi Tunggal (SouthCity).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
+          <t>EXECUTIVE SUMMARY</t>
+        </is>
+      </c>
+      <c r="C15" s="58" t="n"/>
+      <c r="D15" s="58" t="n"/>
+      <c r="E15" s="58" t="n"/>
+      <c r="F15" s="58" t="n"/>
+      <c r="G15" s="58" t="n"/>
+      <c r="H15" s="58" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1" s="31">
       <c r="B16" s="57" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="57" t="inlineStr">
-        <is>
-          <t>**EXECUTIVE SUMMARY**</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="57" t="inlineStr">
-        <is>
-          <t>**Rekonsiliasi Advance Settlement Periode April 2026**</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="57" t="inlineStr">
-        <is>
-          <t>**Kepada Yth. Direksi PT. Setiawan Dwi Tunggal (SouthCity)**</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="57" t="inlineStr">
-        <is>
-          <t>**Dari:** Senior Finance &amp; Automation Controller</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="57" t="inlineStr">
-        <is>
-          <t>**Tanggal:** 02 Mei 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
+          <t>Rekonsiliasi Advance Settlement Periode April 2026</t>
+        </is>
+      </c>
+      <c r="C16" s="58" t="n"/>
+      <c r="D16" s="58" t="n"/>
+      <c r="E16" s="58" t="n"/>
+      <c r="F16" s="58" t="n"/>
+      <c r="G16" s="58" t="n"/>
+      <c r="H16" s="58" t="n"/>
+    </row>
+    <row r="17" ht="20" customHeight="1" s="31">
+      <c r="B17" s="59" t="inlineStr">
+        <is>
+          <t>PT. Setiawan Dwi Tunggal (SouthCity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1" s="31">
+      <c r="B18" s="59" t="inlineStr">
+        <is>
+          <t>Tanggal: 26 April 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1" s="31">
+      <c r="B19" s="59" t="inlineStr">
+        <is>
+          <t>Kepada Yth.: Direksi PT. Setiawan Dwi Tunggal</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1" s="31">
+      <c r="B20" s="59" t="inlineStr">
+        <is>
+          <t>Dari: [Nama Anda], Senior Finance &amp; Automation Controller</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="51" customHeight="1" s="31">
+      <c r="B21" s="59" t="inlineStr">
+        <is>
+          <t>Laporan ini menyajikan hasil rekonsiliasi Advance Settlement untuk periode April 2026, dengan fokus pada kinerja penyelesaian uang muka dan identifikasi saldo outstanding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1" s="31">
       <c r="B22" s="57" t="inlineStr">
         <is>
-          <t>Laporan ini menyajikan ringkasan hasil rekonsiliasi Advance Settlement untuk periode April 2026, mencakup kinerja penyelesaian, sorotan transaksi kunci, dan rekomendasi tindak lanjut.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
+          <t>1. Ringkasan Eksekutif &amp; Kinerja Settlement</t>
+        </is>
+      </c>
+      <c r="C22" s="58" t="n"/>
+      <c r="D22" s="58" t="n"/>
+      <c r="E22" s="58" t="n"/>
+      <c r="F22" s="58" t="n"/>
+      <c r="G22" s="58" t="n"/>
+      <c r="H22" s="58" t="n"/>
+    </row>
+    <row r="23" ht="24" customHeight="1" s="31">
       <c r="B23" s="57" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="58" t="inlineStr">
-        <is>
-          <t>### 1. Ringkasan Eksekutif &amp; Kinerja Settlement</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="57" t="inlineStr">
-        <is>
-          <t>Rekonsiliasi Advance Settlement untuk periode April 2026 telah selesai dilaksanakan. Secara keseluruhan, kinerja penyelesaian uang muka menunjukkan efisiensi yang baik dengan rasio penyelesaian yang tinggi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="57" t="inlineStr">
-        <is>
-          <t>*   **Total Nilai Uang Muka (Advance) Awal:** Rp 570.406.879 (dari 15 transaksi)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="57" t="inlineStr">
-        <is>
-          <t>*   **Total Realisasi / Settlement Masuk:** Rp 463.302.663</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="57" t="inlineStr">
-        <is>
-          <t>*   **Total Sisa Saldo Outstanding:** Rp 107.104.216</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="57" t="inlineStr">
-        <is>
-          <t>*   **Rasio Penyelesaian (Settlement Rate):** 81,22%</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="57" t="inlineStr">
-        <is>
-          <t>*   **Jumlah Transaksi Selesai (Fully Settled):** 14 dari 15 transaksi</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="57" t="inlineStr">
-        <is>
-          <t>Tingkat penyelesaian sebesar 81,22% dan 14 dari 15 transaksi telah diselesaikan penuh menunjukkan pengelolaan advance yang efektif, dengan hanya satu transaksi yang masih memiliki saldo terbuka.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="58" t="inlineStr">
-        <is>
-          <t>### 2. Sorotan Transaksi Kritis &amp; Item Unsettled</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="57" t="inlineStr">
-        <is>
-          <t>Satu-satunya transaksi yang masih memiliki sisa saldo terbuka dan menjadi fokus utama adalah:</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
+          <t>Rekonsiliasi Advance Settlement periode April 2026 telah berhasil diselesaikan. Dari total 15 transaksi uang muka dengan nilai awal Rp 570.406.879, sejumlah Rp 463.302.663 telah berhasil direalisasikan atau diselesaikan. Kinerja penyelesaian ini menunjukkan Rasio Penyelesaian (Settlement Rate) sebesar 81.22%. Secara keseluruhan, 14 dari 15 transaksi telah terselesaikan sepenuhnya, menyisakan satu transaksi dengan saldo parsial.</t>
+        </is>
+      </c>
+      <c r="C23" s="58" t="n"/>
+      <c r="D23" s="58" t="n"/>
+      <c r="E23" s="58" t="n"/>
+      <c r="F23" s="58" t="n"/>
+      <c r="G23" s="58" t="n"/>
+      <c r="H23" s="58" t="n"/>
+    </row>
+    <row r="24" ht="24" customHeight="1" s="31">
+      <c r="B24" s="57" t="inlineStr">
+        <is>
+          <t>2. Sorotan Transaksi Kritis &amp; Item Unsettled</t>
+        </is>
+      </c>
+      <c r="C24" s="58" t="n"/>
+      <c r="D24" s="58" t="n"/>
+      <c r="E24" s="58" t="n"/>
+      <c r="F24" s="58" t="n"/>
+      <c r="G24" s="58" t="n"/>
+      <c r="H24" s="58" t="n"/>
+    </row>
+    <row r="25" ht="34" customHeight="1" s="31">
+      <c r="B25" s="59" t="inlineStr">
+        <is>
+          <t>Sisa saldo outstanding sebesar Rp 107.104.216 seluruhnya berasal dari satu transaksi tunggal:</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1" s="31">
+      <c r="B26" s="59" t="inlineStr">
+        <is>
+          <t>- Nama Transaksi: PEMBAYARAN PBB JV 2 SUMMARECON TAHUN 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1" s="31">
+      <c r="B27" s="59" t="inlineStr">
+        <is>
+          <t>- Voucher Pengajuan Advance: PMT2/BK/2602/0092</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1" s="31">
+      <c r="B28" s="59" t="inlineStr">
+        <is>
+          <t>- Nilai Advance Awal: Rp 422.974.179</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="34" customHeight="1" s="31">
+      <c r="B29" s="59" t="inlineStr">
+        <is>
+          <t>- Realisasi Diterima: Rp 315.869.963 (melalui Voucher Penerimaan BCA1/BM/2604/0069 - Penerimaan Pembayaran PBB MSCM AJB JV 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1" s="31">
+      <c r="B30" s="59" t="inlineStr">
+        <is>
+          <t>- Sisa Saldo Terbuka (Outstanding): Rp 107.104.216</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="34" customHeight="1" s="31">
+      <c r="B31" s="59" t="inlineStr">
+        <is>
+          <t>Penyelesaian parsial ini telah dicatat dan saldo terbuka tersebut memerlukan tindak lanjut lebih lanjut untuk penyelesaian penuh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1" s="31">
+      <c r="B32" s="57" t="inlineStr">
+        <is>
+          <t>3. Penyelesaian Multi-Voucher Sukses</t>
+        </is>
+      </c>
+      <c r="C32" s="58" t="n"/>
+      <c r="D32" s="58" t="n"/>
+      <c r="E32" s="58" t="n"/>
+      <c r="F32" s="58" t="n"/>
+      <c r="G32" s="58" t="n"/>
+      <c r="H32" s="58" t="n"/>
+    </row>
+    <row r="33" ht="85" customHeight="1" s="31">
+      <c r="B33" s="59" t="inlineStr">
+        <is>
+          <t>Perlu dicatat keberhasilan penyelesaian 100% untuk transaksi Multi-Voucher Styling Apartemen (2BR &amp; Studio). Rekonsiliasi untuk transaksi ini, yang melibatkan kombinasi belanja vendor dan retur pengembalian kelebihan dana kas, telah diselesaikan secara akurat dan komprehensif. Hal ini menunjukkan efektivitas proses rekonsiliasi kami dalam menangani transaksi yang kompleks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1" s="31">
       <c r="B34" s="57" t="inlineStr">
         <is>
-          <t>*   **Nama Transaksi:** PEMBAYARAN PBB JV 2 SUMMARECON TAHUN 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="57" t="inlineStr">
-        <is>
-          <t>*   **Voucher Pengajuan Advance:** PMT2/BK/2602/0092</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
+          <t>4. Rekomendasi Tindak Lanjut (Action Plan)</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n"/>
+      <c r="D34" s="58" t="n"/>
+      <c r="E34" s="58" t="n"/>
+      <c r="F34" s="58" t="n"/>
+      <c r="G34" s="58" t="n"/>
+      <c r="H34" s="58" t="n"/>
+    </row>
+    <row r="35" ht="34" customHeight="1" s="31">
+      <c r="B35" s="59" t="inlineStr">
+        <is>
+          <t>Berdasarkan hasil rekonsiliasi ini, kami merekomendasikan beberapa langkah tindak lanjut:</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1" s="31">
       <c r="B36" s="57" t="inlineStr">
         <is>
-          <t>*   **Nilai Advance Awal:** Rp 422.974.179</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
+          <t>1.  Tindak Lanjut Saldo Outstanding PBB JV 2 Summarecon: Divisi Finance akan segera berkoordinasi dengan departemen terkait atau pihak JV untuk mempercepat penyelesaian sisa saldo Rp 107.104.216 dari transaksi PBB JV 2 Summarecon. Target penyelesaian penuh akan ditetapkan dalam waktu dekat.</t>
+        </is>
+      </c>
+      <c r="C36" s="58" t="n"/>
+      <c r="D36" s="58" t="n"/>
+      <c r="E36" s="58" t="n"/>
+      <c r="F36" s="58" t="n"/>
+      <c r="G36" s="58" t="n"/>
+      <c r="H36" s="58" t="n"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" s="31">
       <c r="B37" s="57" t="inlineStr">
         <is>
-          <t>*   **Realisasi Diterima (Parsial):** Rp 315.869.963 (melalui voucher BCA1/BM/2604/0069 - Penerimaan Pembayaran PBB MSCM AJB JV 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
+          <t>2.  Evaluasi Proses Settlement: Mengevaluasi potensi percepatan proses settlement untuk transaksi advance dengan nilai besar, guna meminimalkan durasi saldo outstanding di masa mendatang.</t>
+        </is>
+      </c>
+      <c r="C37" s="58" t="n"/>
+      <c r="D37" s="58" t="n"/>
+      <c r="E37" s="58" t="n"/>
+      <c r="F37" s="58" t="n"/>
+      <c r="G37" s="58" t="n"/>
+      <c r="H37" s="58" t="n"/>
+    </row>
+    <row r="38" ht="24" customHeight="1" s="31">
       <c r="B38" s="57" t="inlineStr">
         <is>
-          <t>*   **Sisa Saldo Terbuka:** Rp 107.104.216</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="57" t="inlineStr">
-        <is>
-          <t>Sisa saldo ini merupakan hasil dari pelunasan parsial atas pembayaran PBB JV 2 Summarecon, di mana sebagian dana telah diterima kembali, namun masih terdapat selisih yang belum terselesaikan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="58" t="inlineStr">
-        <is>
-          <t>### 3. Penyelesaian Multi-Voucher Sukses</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="57" t="inlineStr">
-        <is>
-          <t>Kami juga ingin menyoroti keberhasilan penyelesaian 100% atas transaksi **Multi-Voucher Styling Apartemen (2BR &amp; Studio)**. Rekonsiliasi untuk transaksi ini, yang melibatkan kombinasi belanja vendor dan retur pengembalian kelebihan dana kas, telah diselesaikan secara akurat dan komprehensif. Hal ini menunjukkan kemampuan tim dalam menangani transaksi yang kompleks dengan berbagai sumber penyelesaian.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="58" t="inlineStr">
-        <is>
-          <t>### 4. Rekomendasi Tindak Lanjut (Action Plan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="57" t="inlineStr">
-        <is>
-          <t>Berdasarkan hasil rekonsiliasi ini, kami merekomendasikan langkah-langkah berikut:</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="57" t="inlineStr">
-        <is>
-          <t>1.  **Tindak Lanjut Saldo PBB JV 2 Summarecon:** Segera lakukan koordinasi dan tindak lanjut dengan departemen terkait atau mitra JV untuk mengklarifikasi dan menyelesaikan sisa saldo Rp 107.104.216 dari transaksi PBB JV 2 Summarecon. Target penyelesaian diharapkan dalam 2 minggu ke depan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="57" t="inlineStr">
-        <is>
-          <t>2.  **Analisis Akar Masalah (Opsional):** Identifikasi penyebab sisa saldo PBB JV 2 Summarecon untuk mencegah kejadian serupa di masa mendatang, jika memungkinkan, atau untuk memastikan proses settlement di masa depan lebih efisien.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="57" t="inlineStr">
-        <is>
-          <t>3.  **Pemantauan Berkelanjutan:** Terus tingkatkan pemantauan dan percepatan proses settlement untuk menjaga rasio penyelesaian yang tinggi dan meminimalkan saldo outstanding secara proaktif.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="57" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="57" t="inlineStr">
-        <is>
-          <t>Demikian Executive Summary ini kami sampaikan untuk menjadi perhatian dan tindak lanjut Direksi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="57" t="inlineStr">
+          <t>3.  Pemanfaatan Otomatisasi: Mempertimbangkan implementasi sistem notifikasi otomatis atau reminder untuk transaksi advance yang mendekati jatuh tempo settlement, khususnya untuk transaksi parsial, guna meningkatkan efisiensi dan akurasi pelacakan.</t>
+        </is>
+      </c>
+      <c r="C38" s="58" t="n"/>
+      <c r="D38" s="58" t="n"/>
+      <c r="E38" s="58" t="n"/>
+      <c r="F38" s="58" t="n"/>
+      <c r="G38" s="58" t="n"/>
+      <c r="H38" s="58" t="n"/>
+    </row>
+    <row r="39" ht="20" customHeight="1" s="31">
+      <c r="B39" s="59" t="inlineStr">
         <is>
           <t>Hormat kami,</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="B50" s="57" t="inlineStr">
-        <is>
-          <t>**[Nama Anda]**</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="57" t="inlineStr">
+    <row r="40" ht="20" customHeight="1" s="31">
+      <c r="B40" s="59" t="inlineStr">
+        <is>
+          <t>[Nama Anda]</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1" s="31">
+      <c r="B41" s="59" t="inlineStr">
         <is>
           <t>Senior Finance &amp; Automation Controller</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="B52" s="57" t="inlineStr">
+    <row r="42" ht="20" customHeight="1" s="31">
+      <c r="B42" s="59" t="inlineStr">
         <is>
           <t>PT. Setiawan Dwi Tunggal (SouthCity)</t>
         </is>
       </c>
     </row>
+    <row r="43" ht="15" customHeight="1" s="31"/>
   </sheetData>
-  <mergeCells count="48">
+  <mergeCells count="38">
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="B40:H40"/>
-    <mergeCell ref="B49:H49"/>
     <mergeCell ref="B24:H24"/>
     <mergeCell ref="B30:H30"/>
     <mergeCell ref="B15:H15"/>
     <mergeCell ref="B33:H33"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B51:H51"/>
     <mergeCell ref="B20:H20"/>
     <mergeCell ref="B37:H37"/>
-    <mergeCell ref="B45:H45"/>
     <mergeCell ref="B36:H36"/>
     <mergeCell ref="B32:H32"/>
-    <mergeCell ref="B50:H50"/>
     <mergeCell ref="B26:H26"/>
     <mergeCell ref="B41:H41"/>
     <mergeCell ref="B35:H35"/>
     <mergeCell ref="F5:G5"/>
-    <mergeCell ref="B47:H47"/>
     <mergeCell ref="B16:H16"/>
     <mergeCell ref="B25:H25"/>
     <mergeCell ref="B31:H31"/>
-    <mergeCell ref="B46:H46"/>
     <mergeCell ref="B22:H22"/>
     <mergeCell ref="B18:H18"/>
     <mergeCell ref="B27:H27"/>
-    <mergeCell ref="B52:H52"/>
     <mergeCell ref="B21:H21"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B43:H43"/>
     <mergeCell ref="B39:H39"/>
-    <mergeCell ref="B48:H48"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="B42:H42"/>
     <mergeCell ref="B7:D7"/>
@@ -1266,7 +1249,6 @@
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="B13:H13"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B44:H44"/>
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="B38:H38"/>
     <mergeCell ref="B29:H29"/>

</xml_diff>

<commit_message>
feat: improve Excel column widths, layout padding, and clean output formatting
</commit_message>
<xml_diff>
--- a/output/Working_Paper_Result.xlsx
+++ b/output/Working_Paper_Result.xlsx
@@ -135,7 +135,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="34">
     <border/>
     <border>
       <bottom style="medium">
@@ -423,11 +423,43 @@
         <color rgb="00CBD5E0"/>
       </bottom>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00CBD5E0"/>
+      </top>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="00CBD5E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E0"/>
+      </top>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="00CBD5E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E0"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00CBD5E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -526,13 +558,14 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -540,6 +573,8 @@
     <xf numFmtId="0" fontId="12" fillId="5" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -549,6 +584,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -825,437 +863,519 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" style="31" min="1" max="1"/>
+    <col width="18" customWidth="1" style="31" min="2" max="2"/>
+    <col width="16" customWidth="1" style="31" min="3" max="3"/>
+    <col width="14" customWidth="1" style="31" min="4" max="4"/>
+    <col width="18" customWidth="1" style="31" min="5" max="5"/>
+    <col width="16" customWidth="1" style="31" min="6" max="6"/>
+    <col width="16" customWidth="1" style="31" min="7" max="7"/>
+    <col width="16" customWidth="1" style="31" min="8" max="8"/>
+    <col width="14" customWidth="1" style="31" min="9" max="9"/>
+    <col width="14" customWidth="1" style="31" min="10" max="10"/>
+    <col width="12" customWidth="1" style="31" min="11" max="11"/>
+    <col width="12" customWidth="1" style="31" min="12" max="12"/>
+  </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" s="31">
+    <row r="1" ht="36" customHeight="1" s="31">
       <c r="A1" s="49" t="inlineStr">
         <is>
           <t>SOUTHCITY FINANCE &amp; IT AUTOMATION — ADVANCE SETTLEMENT DASHBOARD</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" s="31">
-      <c r="A2" s="50" t="inlineStr">
+      <c r="B1" s="50" t="n"/>
+      <c r="C1" s="50" t="n"/>
+      <c r="D1" s="50" t="n"/>
+      <c r="E1" s="50" t="n"/>
+      <c r="F1" s="50" t="n"/>
+      <c r="G1" s="50" t="n"/>
+      <c r="H1" s="50" t="n"/>
+      <c r="I1" s="50" t="n"/>
+      <c r="J1" s="50" t="n"/>
+      <c r="K1" s="50" t="n"/>
+      <c r="L1" s="50" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" s="31">
+      <c r="A2" s="51" t="inlineStr">
         <is>
           <t>Executive Reconciliation Report | Periode: April 2026 | Total Settlement Rate: 81.22%</t>
         </is>
       </c>
+      <c r="B2" s="50" t="n"/>
+      <c r="C2" s="50" t="n"/>
+      <c r="D2" s="50" t="n"/>
+      <c r="E2" s="50" t="n"/>
+      <c r="F2" s="50" t="n"/>
+      <c r="G2" s="50" t="n"/>
+      <c r="H2" s="50" t="n"/>
+      <c r="I2" s="50" t="n"/>
+      <c r="J2" s="50" t="n"/>
+      <c r="K2" s="50" t="n"/>
+      <c r="L2" s="50" t="n"/>
     </row>
     <row r="3" ht="10" customHeight="1" s="31"/>
-    <row r="4">
-      <c r="B4" s="51" t="inlineStr">
+    <row r="4" ht="22" customHeight="1" s="31">
+      <c r="B4" s="52" t="inlineStr">
         <is>
           <t>TOTAL ADVANCE</t>
         </is>
       </c>
-      <c r="C4" s="52" t="n"/>
-      <c r="D4" s="51" t="inlineStr">
+      <c r="C4" s="53" t="n"/>
+      <c r="D4" s="53" t="n"/>
+      <c r="E4" s="52" t="inlineStr">
         <is>
           <t>TOTAL REALISASI</t>
         </is>
       </c>
-      <c r="E4" s="52" t="n"/>
-      <c r="F4" s="51" t="inlineStr">
+      <c r="F4" s="53" t="n"/>
+      <c r="G4" s="53" t="n"/>
+      <c r="H4" s="52" t="inlineStr">
         <is>
           <t>SISA SALDO (OUTSTANDING)</t>
         </is>
       </c>
-      <c r="G4" s="52" t="n"/>
-    </row>
-    <row r="5">
-      <c r="B5" s="53" t="inlineStr">
+      <c r="I4" s="53" t="n"/>
+      <c r="J4" s="53" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1" s="31">
+      <c r="B5" s="54" t="inlineStr">
         <is>
           <t>Rp 570,406,879</t>
         </is>
       </c>
-      <c r="C5" s="52" t="n"/>
-      <c r="D5" s="53" t="inlineStr">
+      <c r="C5" s="53" t="n"/>
+      <c r="D5" s="53" t="n"/>
+      <c r="E5" s="54" t="inlineStr">
         <is>
           <t>Rp 463,302,663</t>
         </is>
       </c>
-      <c r="E5" s="52" t="n"/>
-      <c r="F5" s="53" t="inlineStr">
+      <c r="F5" s="53" t="n"/>
+      <c r="G5" s="53" t="n"/>
+      <c r="H5" s="54" t="inlineStr">
         <is>
           <t>Rp 107,104,216</t>
         </is>
       </c>
-      <c r="G5" s="52" t="n"/>
+      <c r="I5" s="53" t="n"/>
+      <c r="J5" s="53" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="54" t="inlineStr">
+      <c r="B7" s="55" t="inlineStr">
         <is>
           <t>RINGKASAN STATUS TRANSAKSI</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="55" t="inlineStr">
+      <c r="B8" s="56" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C8" s="55" t="inlineStr">
+      <c r="C8" s="57" t="n"/>
+      <c r="D8" s="56" t="inlineStr">
         <is>
           <t>Jumlah Item</t>
         </is>
       </c>
-      <c r="D8" s="55" t="inlineStr">
+      <c r="E8" s="56" t="inlineStr">
         <is>
           <t>Keterangan</t>
         </is>
       </c>
+      <c r="F8" s="57" t="n"/>
+      <c r="G8" s="57" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="52" t="inlineStr">
+      <c r="B9" s="58" t="inlineStr">
         <is>
           <t>Fully Settled (Lunas)</t>
         </is>
       </c>
-      <c r="C9" s="56" t="n">
+      <c r="C9" s="58" t="n"/>
+      <c r="D9" s="59" t="n">
         <v>14</v>
       </c>
-      <c r="D9" s="52" t="inlineStr">
+      <c r="E9" s="58" t="inlineStr">
         <is>
           <t>100% Selesai &amp; Cocok dengan GL</t>
         </is>
       </c>
+      <c r="F9" s="58" t="n"/>
+      <c r="G9" s="58" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="52" t="inlineStr">
+      <c r="B10" s="58" t="inlineStr">
         <is>
           <t>Partially Settled (Sebagian)</t>
         </is>
       </c>
-      <c r="C10" s="56" t="n">
+      <c r="C10" s="58" t="n"/>
+      <c r="D10" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="52" t="inlineStr">
+      <c r="E10" s="58" t="inlineStr">
         <is>
           <t>PBB JV 2 Summarecon (Sisa Rp 107.1M)</t>
         </is>
       </c>
+      <c r="F10" s="58" t="n"/>
+      <c r="G10" s="58" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="52" t="inlineStr">
+      <c r="B11" s="58" t="inlineStr">
         <is>
           <t>Unsettled (Belum Selesai)</t>
         </is>
       </c>
-      <c r="C11" s="56" t="n">
+      <c r="C11" s="58" t="n"/>
+      <c r="D11" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="52" t="inlineStr">
+      <c r="E11" s="58" t="inlineStr">
         <is>
           <t>Tidak ada transaksi tanpa matching</t>
         </is>
       </c>
+      <c r="F11" s="58" t="n"/>
+      <c r="G11" s="58" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="54" t="inlineStr">
+      <c r="B13" s="55" t="inlineStr">
         <is>
           <t>EXECUTIVE SUMMARY (LAPORAN REKONSILIASI)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1" s="31">
-      <c r="B15" s="57" t="inlineStr">
-        <is>
-          <t>EXECUTIVE SUMMARY</t>
-        </is>
-      </c>
-      <c r="C15" s="58" t="n"/>
-      <c r="D15" s="58" t="n"/>
-      <c r="E15" s="58" t="n"/>
-      <c r="F15" s="58" t="n"/>
-      <c r="G15" s="58" t="n"/>
-      <c r="H15" s="58" t="n"/>
-    </row>
-    <row r="16" ht="24" customHeight="1" s="31">
-      <c r="B16" s="57" t="inlineStr">
-        <is>
-          <t>Rekonsiliasi Advance Settlement Periode April 2026</t>
-        </is>
-      </c>
-      <c r="C16" s="58" t="n"/>
-      <c r="D16" s="58" t="n"/>
-      <c r="E16" s="58" t="n"/>
-      <c r="F16" s="58" t="n"/>
-      <c r="G16" s="58" t="n"/>
-      <c r="H16" s="58" t="n"/>
+      <c r="B15" s="60" t="inlineStr">
+        <is>
+          <t>EXECUTIVE SUMMARY: REKONSILIASI ADVANCE SETTLEMENT</t>
+        </is>
+      </c>
+      <c r="C15" s="61" t="n"/>
+      <c r="D15" s="61" t="n"/>
+      <c r="E15" s="61" t="n"/>
+      <c r="F15" s="61" t="n"/>
+      <c r="G15" s="61" t="n"/>
+      <c r="H15" s="61" t="n"/>
+      <c r="I15" s="61" t="n"/>
+      <c r="J15" s="61" t="n"/>
+      <c r="K15" s="61" t="n"/>
+      <c r="L15" s="61" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1" s="31">
+      <c r="B16" s="62" t="inlineStr">
+        <is>
+          <t>Periode: April 2026</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1" s="31">
-      <c r="B17" s="59" t="inlineStr">
-        <is>
-          <t>PT. Setiawan Dwi Tunggal (SouthCity)</t>
+      <c r="B17" s="62" t="inlineStr">
+        <is>
+          <t>Entitas: PT. Setiawan Dwi Tunggal (SouthCity)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" s="31">
-      <c r="B18" s="59" t="inlineStr">
-        <is>
-          <t>Tanggal: 26 April 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1" s="31">
-      <c r="B19" s="59" t="inlineStr">
-        <is>
-          <t>Kepada Yth.: Direksi PT. Setiawan Dwi Tunggal</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1" s="31">
-      <c r="B20" s="59" t="inlineStr">
-        <is>
-          <t>Dari: [Nama Anda], Senior Finance &amp; Automation Controller</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="51" customHeight="1" s="31">
-      <c r="B21" s="59" t="inlineStr">
-        <is>
-          <t>Laporan ini menyajikan hasil rekonsiliasi Advance Settlement untuk periode April 2026, dengan fokus pada kinerja penyelesaian uang muka dan identifikasi saldo outstanding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1" s="31">
-      <c r="B22" s="57" t="inlineStr">
+      <c r="B18" s="62" t="inlineStr">
+        <is>
+          <t>Disusun oleh: Senior Finance &amp; Automation Controller</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1" s="31">
+      <c r="B19" s="60" t="inlineStr">
         <is>
           <t>1. Ringkasan Eksekutif &amp; Kinerja Settlement</t>
         </is>
       </c>
-      <c r="C22" s="58" t="n"/>
-      <c r="D22" s="58" t="n"/>
-      <c r="E22" s="58" t="n"/>
-      <c r="F22" s="58" t="n"/>
-      <c r="G22" s="58" t="n"/>
-      <c r="H22" s="58" t="n"/>
-    </row>
-    <row r="23" ht="24" customHeight="1" s="31">
-      <c r="B23" s="57" t="inlineStr">
-        <is>
-          <t>Rekonsiliasi Advance Settlement periode April 2026 telah berhasil diselesaikan. Dari total 15 transaksi uang muka dengan nilai awal Rp 570.406.879, sejumlah Rp 463.302.663 telah berhasil direalisasikan atau diselesaikan. Kinerja penyelesaian ini menunjukkan Rasio Penyelesaian (Settlement Rate) sebesar 81.22%. Secara keseluruhan, 14 dari 15 transaksi telah terselesaikan sepenuhnya, menyisakan satu transaksi dengan saldo parsial.</t>
-        </is>
-      </c>
-      <c r="C23" s="58" t="n"/>
-      <c r="D23" s="58" t="n"/>
-      <c r="E23" s="58" t="n"/>
-      <c r="F23" s="58" t="n"/>
-      <c r="G23" s="58" t="n"/>
-      <c r="H23" s="58" t="n"/>
-    </row>
-    <row r="24" ht="24" customHeight="1" s="31">
-      <c r="B24" s="57" t="inlineStr">
+      <c r="C19" s="61" t="n"/>
+      <c r="D19" s="61" t="n"/>
+      <c r="E19" s="61" t="n"/>
+      <c r="F19" s="61" t="n"/>
+      <c r="G19" s="61" t="n"/>
+      <c r="H19" s="61" t="n"/>
+      <c r="I19" s="61" t="n"/>
+      <c r="J19" s="61" t="n"/>
+      <c r="K19" s="61" t="n"/>
+      <c r="L19" s="61" t="n"/>
+    </row>
+    <row r="20" ht="51" customHeight="1" s="31">
+      <c r="B20" s="62" t="inlineStr">
+        <is>
+          <t>Proses rekonsiliasi Advance Settlement periode April 2026 telah diselesaikan dengan hasil yang sangat baik. Dari total 15 transaksi advance yang tercatat, sebanyak 14 transaksi telah berhasil diselesaikan (fully settled0, mencerminkan efisiensi operasional dan kepatuhan administratif yang tinggi di lini departemen terkait.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" s="31">
+      <c r="B21" s="63" t="inlineStr">
+        <is>
+          <t>- Total Nilai Uang Muka (Advance) Awal: Rp 570,406,879 (15 Transaksi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1" s="31">
+      <c r="B22" s="63" t="inlineStr">
+        <is>
+          <t>- Total Realisasi / Settlement Masuk: Rp 463,302,663</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1" s="31">
+      <c r="B23" s="63" t="inlineStr">
+        <is>
+          <t>- Total Sisa Saldo Outstanding: Rp 107,104,216</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1" s="31">
+      <c r="B24" s="63" t="inlineStr">
+        <is>
+          <t>- Rasio Penyelesaian (Settlement Rate): 81.22%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1" s="31">
+      <c r="B25" s="63" t="inlineStr">
+        <is>
+          <t>- Status Transaksi: 14 Selesai / 1 Berjalan (Partial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1" s="31">
+      <c r="B26" s="60" t="inlineStr">
         <is>
           <t>2. Sorotan Transaksi Kritis &amp; Item Unsettled</t>
         </is>
       </c>
-      <c r="C24" s="58" t="n"/>
-      <c r="D24" s="58" t="n"/>
-      <c r="E24" s="58" t="n"/>
-      <c r="F24" s="58" t="n"/>
-      <c r="G24" s="58" t="n"/>
-      <c r="H24" s="58" t="n"/>
-    </row>
-    <row r="25" ht="34" customHeight="1" s="31">
-      <c r="B25" s="59" t="inlineStr">
-        <is>
-          <t>Sisa saldo outstanding sebesar Rp 107.104.216 seluruhnya berasal dari satu transaksi tunggal:</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1" s="31">
-      <c r="B26" s="59" t="inlineStr">
-        <is>
-          <t>- Nama Transaksi: PEMBAYARAN PBB JV 2 SUMMARECON TAHUN 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1" s="31">
-      <c r="B27" s="59" t="inlineStr">
-        <is>
-          <t>- Voucher Pengajuan Advance: PMT2/BK/2602/0092</t>
+      <c r="C26" s="61" t="n"/>
+      <c r="D26" s="61" t="n"/>
+      <c r="E26" s="61" t="n"/>
+      <c r="F26" s="61" t="n"/>
+      <c r="G26" s="61" t="n"/>
+      <c r="H26" s="61" t="n"/>
+      <c r="I26" s="61" t="n"/>
+      <c r="J26" s="61" t="n"/>
+      <c r="K26" s="61" t="n"/>
+      <c r="L26" s="61" t="n"/>
+    </row>
+    <row r="27" ht="34" customHeight="1" s="31">
+      <c r="B27" s="62" t="inlineStr">
+        <is>
+          <t>Meskipun mayoritas transaksi telah ditutup, terdapat satu item material bernilai tinggi yang masih menyisakan saldo outstanding:</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1" s="31">
-      <c r="B28" s="59" t="inlineStr">
-        <is>
-          <t>- Nilai Advance Awal: Rp 422.974.179</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="34" customHeight="1" s="31">
-      <c r="B29" s="59" t="inlineStr">
-        <is>
-          <t>- Realisasi Diterima: Rp 315.869.963 (melalui Voucher Penerimaan BCA1/BM/2604/0069 - Penerimaan Pembayaran PBB MSCM AJB JV 2)</t>
+      <c r="B28" s="63" t="inlineStr">
+        <is>
+          <t>- Deskripsi Item: Pembayaran PBB JV 2 Summarecon Tahun 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1" s="31">
+      <c r="B29" s="63" t="inlineStr">
+        <is>
+          <t>- Nomor Voucher Pengajuan: PMT2/BK/2602/0092</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" s="31">
-      <c r="B30" s="59" t="inlineStr">
-        <is>
-          <t>- Sisa Saldo Terbuka (Outstanding): Rp 107.104.216</t>
+      <c r="B30" s="63" t="inlineStr">
+        <is>
+          <t>- Nilai Advance Awal: Rp 422,974,179</t>
         </is>
       </c>
     </row>
     <row r="31" ht="34" customHeight="1" s="31">
-      <c r="B31" s="59" t="inlineStr">
-        <is>
-          <t>Penyelesaian parsial ini telah dicatat dan saldo terbuka tersebut memerlukan tindak lanjut lebih lanjut untuk penyelesaian penuh.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="24" customHeight="1" s="31">
-      <c r="B32" s="57" t="inlineStr">
-        <is>
-          <t>3. Penyelesaian Multi-Voucher Sukses</t>
-        </is>
-      </c>
-      <c r="C32" s="58" t="n"/>
-      <c r="D32" s="58" t="n"/>
-      <c r="E32" s="58" t="n"/>
-      <c r="F32" s="58" t="n"/>
-      <c r="G32" s="58" t="n"/>
-      <c r="H32" s="58" t="n"/>
-    </row>
-    <row r="33" ht="85" customHeight="1" s="31">
-      <c r="B33" s="59" t="inlineStr">
-        <is>
-          <t>Perlu dicatat keberhasilan penyelesaian 100% untuk transaksi Multi-Voucher Styling Apartemen (2BR &amp; Studio). Rekonsiliasi untuk transaksi ini, yang melibatkan kombinasi belanja vendor dan retur pengembalian kelebihan dana kas, telah diselesaikan secara akurat dan komprehensif. Hal ini menunjukkan efektivitas proses rekonsiliasi kami dalam menangani transaksi yang kompleks.</t>
+      <c r="B31" s="63" t="inlineStr">
+        <is>
+          <t>- Realisasi Diterima: Rp 315,869,963 (Ref. Voucher Penerimaan: BCA1/BM/2604/0069 - Penerimaan Pembayaran PBB MSCM AJB JV 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1" s="31">
+      <c r="B32" s="63" t="inlineStr">
+        <is>
+          <t>- Sisa Saldo Terbuka (Outstanding): Rp 107,104,216</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="34" customHeight="1" s="31">
+      <c r="B33" s="62" t="inlineStr">
+        <is>
+          <t>Catatan Analis: Sisa saldo sebesar Rp 107.104.216 memerlukan monitoring ketat karena menyerap porsi terbesar dari total outstanding bulan ini.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="24" customHeight="1" s="31">
-      <c r="B34" s="57" t="inlineStr">
+      <c r="B34" s="60" t="inlineStr">
+        <is>
+          <t>3. Penyelesaian Multi-Voucher Sukses (Styling Apartemen)</t>
+        </is>
+      </c>
+      <c r="C34" s="61" t="n"/>
+      <c r="D34" s="61" t="n"/>
+      <c r="E34" s="61" t="n"/>
+      <c r="F34" s="61" t="n"/>
+      <c r="G34" s="61" t="n"/>
+      <c r="H34" s="61" t="n"/>
+      <c r="I34" s="61" t="n"/>
+      <c r="J34" s="61" t="n"/>
+      <c r="K34" s="61" t="n"/>
+      <c r="L34" s="61" t="n"/>
+    </row>
+    <row r="35" ht="34" customHeight="1" s="31">
+      <c r="B35" s="62" t="inlineStr">
+        <is>
+          <t>Sebagai catatan positif dalam siklus rekonsiliasi periode ini, seluruh rangkaian transaksi Multi-Voucher untuk proyek Styling Apartemen (tipe 2BR &amp; Studio) telah berhasil diselesaikan 100% secara akurat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="34" customHeight="1" s="31">
+      <c r="B36" s="62" t="inlineStr">
+        <is>
+          <t>Rekonsiliasi komprehensif ini sukses memetakan pencocokan silang yang kompleks antara pembayaran ke vendor dan pengembalian sisa kelebihan dana kas (retur), tanpa ditemukan selisih pencatatan (zero discrepancy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1" s="31">
+      <c r="B37" s="60" t="inlineStr">
         <is>
           <t>4. Rekomendasi Tindak Lanjut (Action Plan)</t>
         </is>
       </c>
-      <c r="C34" s="58" t="n"/>
-      <c r="D34" s="58" t="n"/>
-      <c r="E34" s="58" t="n"/>
-      <c r="F34" s="58" t="n"/>
-      <c r="G34" s="58" t="n"/>
-      <c r="H34" s="58" t="n"/>
-    </row>
-    <row r="35" ht="34" customHeight="1" s="31">
-      <c r="B35" s="59" t="inlineStr">
-        <is>
-          <t>Berdasarkan hasil rekonsiliasi ini, kami merekomendasikan beberapa langkah tindak lanjut:</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="24" customHeight="1" s="31">
-      <c r="B36" s="57" t="inlineStr">
-        <is>
-          <t>1.  Tindak Lanjut Saldo Outstanding PBB JV 2 Summarecon: Divisi Finance akan segera berkoordinasi dengan departemen terkait atau pihak JV untuk mempercepat penyelesaian sisa saldo Rp 107.104.216 dari transaksi PBB JV 2 Summarecon. Target penyelesaian penuh akan ditetapkan dalam waktu dekat.</t>
-        </is>
-      </c>
-      <c r="C36" s="58" t="n"/>
-      <c r="D36" s="58" t="n"/>
-      <c r="E36" s="58" t="n"/>
-      <c r="F36" s="58" t="n"/>
-      <c r="G36" s="58" t="n"/>
-      <c r="H36" s="58" t="n"/>
-    </row>
-    <row r="37" ht="24" customHeight="1" s="31">
-      <c r="B37" s="57" t="inlineStr">
-        <is>
-          <t>2.  Evaluasi Proses Settlement: Mengevaluasi potensi percepatan proses settlement untuk transaksi advance dengan nilai besar, guna meminimalkan durasi saldo outstanding di masa mendatang.</t>
-        </is>
-      </c>
-      <c r="C37" s="58" t="n"/>
-      <c r="D37" s="58" t="n"/>
-      <c r="E37" s="58" t="n"/>
-      <c r="F37" s="58" t="n"/>
-      <c r="G37" s="58" t="n"/>
-      <c r="H37" s="58" t="n"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" s="31">
-      <c r="B38" s="57" t="inlineStr">
-        <is>
-          <t>3.  Pemanfaatan Otomatisasi: Mempertimbangkan implementasi sistem notifikasi otomatis atau reminder untuk transaksi advance yang mendekati jatuh tempo settlement, khususnya untuk transaksi parsial, guna meningkatkan efisiensi dan akurasi pelacakan.</t>
-        </is>
-      </c>
-      <c r="C38" s="58" t="n"/>
-      <c r="D38" s="58" t="n"/>
-      <c r="E38" s="58" t="n"/>
-      <c r="F38" s="58" t="n"/>
-      <c r="G38" s="58" t="n"/>
-      <c r="H38" s="58" t="n"/>
-    </row>
-    <row r="39" ht="20" customHeight="1" s="31">
-      <c r="B39" s="59" t="inlineStr">
-        <is>
-          <t>Hormat kami,</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1" s="31">
-      <c r="B40" s="59" t="inlineStr">
-        <is>
-          <t>[Nama Anda]</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1" s="31">
-      <c r="B41" s="59" t="inlineStr">
-        <is>
-          <t>Senior Finance &amp; Automation Controller</t>
-        </is>
-      </c>
+      <c r="C37" s="61" t="n"/>
+      <c r="D37" s="61" t="n"/>
+      <c r="E37" s="61" t="n"/>
+      <c r="F37" s="61" t="n"/>
+      <c r="G37" s="61" t="n"/>
+      <c r="H37" s="61" t="n"/>
+      <c r="I37" s="61" t="n"/>
+      <c r="J37" s="61" t="n"/>
+      <c r="K37" s="61" t="n"/>
+      <c r="L37" s="61" t="n"/>
+    </row>
+    <row r="38" ht="34" customHeight="1" s="31">
+      <c r="B38" s="62" t="inlineStr">
+        <is>
+          <t>Untuk menjaga akuntabilitas keuangan dan mempercepat penutupan buku periode selanjutnya, berikut adalah langkah taktis yang direkomendasikan bagi tim Finance dan manajemen:</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1" s="31">
+      <c r="B39" s="60" t="inlineStr">
+        <is>
+          <t>1. Penagihan &amp; Konfirmasi PBB JV 2 Summarecon: Tim Finance diinstruksikan untuk segera berkoordinasi dengan pihak terkait guna memastikan jadwal pelunasan sisa saldo outstanding sebesar Rp 107,104,216, serta memastikan kelengkapan dokumen pendukung untuk pencatatan full settlement pada siklus berikutnya.</t>
+        </is>
+      </c>
+      <c r="C39" s="61" t="n"/>
+      <c r="D39" s="61" t="n"/>
+      <c r="E39" s="61" t="n"/>
+      <c r="F39" s="61" t="n"/>
+      <c r="G39" s="61" t="n"/>
+      <c r="H39" s="61" t="n"/>
+      <c r="I39" s="61" t="n"/>
+      <c r="J39" s="61" t="n"/>
+      <c r="K39" s="61" t="n"/>
+      <c r="L39" s="61" t="n"/>
+    </row>
+    <row r="40" ht="24" customHeight="1" s="31">
+      <c r="B40" s="60" t="inlineStr">
+        <is>
+          <t>2. Automasi Modul Advance: Memanfaatkan modul automation pada sistem keuangan SouthCity guna memonitor umur advance (aging of advances), sehingga potensi outstanding jangka panjang dapat terdeteksi lebih dini.</t>
+        </is>
+      </c>
+      <c r="C40" s="61" t="n"/>
+      <c r="D40" s="61" t="n"/>
+      <c r="E40" s="61" t="n"/>
+      <c r="F40" s="61" t="n"/>
+      <c r="G40" s="61" t="n"/>
+      <c r="H40" s="61" t="n"/>
+      <c r="I40" s="61" t="n"/>
+      <c r="J40" s="61" t="n"/>
+      <c r="K40" s="61" t="n"/>
+      <c r="L40" s="61" t="n"/>
+    </row>
+    <row r="41" ht="24" customHeight="1" s="31">
+      <c r="B41" s="60" t="inlineStr">
+        <is>
+          <t>3. Standarisasi Proses Multi-Voucher: Menjadikan keberhasilan rekonsiliasi Styling Apartemen sebagai benchmark (standar operasional prosedur) untuk penanganan proyek-proyek multi-vendor di masa mendatang.</t>
+        </is>
+      </c>
+      <c r="C41" s="61" t="n"/>
+      <c r="D41" s="61" t="n"/>
+      <c r="E41" s="61" t="n"/>
+      <c r="F41" s="61" t="n"/>
+      <c r="G41" s="61" t="n"/>
+      <c r="H41" s="61" t="n"/>
+      <c r="I41" s="61" t="n"/>
+      <c r="J41" s="61" t="n"/>
+      <c r="K41" s="61" t="n"/>
+      <c r="L41" s="61" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1" s="31">
-      <c r="B42" s="59" t="inlineStr">
-        <is>
-          <t>PT. Setiawan Dwi Tunggal (SouthCity)</t>
+      <c r="B42" s="62" t="inlineStr">
+        <is>
+          <t>Dokumen ini bersifat rahasia dan ditujukan khusus untuk laporan internal kepada Direksi PT. Setiawan Dwi Tunggal.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="31"/>
   </sheetData>
-  <mergeCells count="38">
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="B40:H40"/>
-    <mergeCell ref="B24:H24"/>
-    <mergeCell ref="B30:H30"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B33:H33"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B20:H20"/>
-    <mergeCell ref="B37:H37"/>
-    <mergeCell ref="B36:H36"/>
-    <mergeCell ref="B32:H32"/>
-    <mergeCell ref="B26:H26"/>
-    <mergeCell ref="B41:H41"/>
-    <mergeCell ref="B35:H35"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B25:H25"/>
-    <mergeCell ref="B31:H31"/>
-    <mergeCell ref="B22:H22"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B27:H27"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B39:H39"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="B42:H42"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B23:H23"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="B38:H38"/>
-    <mergeCell ref="B29:H29"/>
-    <mergeCell ref="B19:H19"/>
-    <mergeCell ref="B34:H34"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B28:H28"/>
+  <mergeCells count="46">
+    <mergeCell ref="B35:L35"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="B26:L26"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B16:L16"/>
+    <mergeCell ref="B25:L25"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="B22:L22"/>
+    <mergeCell ref="B31:L31"/>
+    <mergeCell ref="B18:L18"/>
+    <mergeCell ref="B27:L27"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B21:L21"/>
+    <mergeCell ref="B39:L39"/>
+    <mergeCell ref="B42:L42"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="B23:L23"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B13:L13"/>
+    <mergeCell ref="B38:L38"/>
+    <mergeCell ref="B29:L29"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B19:L19"/>
+    <mergeCell ref="B34:L34"/>
+    <mergeCell ref="B37:L37"/>
+    <mergeCell ref="B28:L28"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="B30:L30"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B15:L15"/>
+    <mergeCell ref="B33:L33"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="B24:L24"/>
+    <mergeCell ref="B20:L20"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="B32:L32"/>
+    <mergeCell ref="B41:L41"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>